<commit_message>
Fotos en los eventos (columna Foto de la hoja)
Acepta enlaces de Google Drive o direcciones directas de imágenes. Si la
foto no se puede cargar, la tarjeta se muestra sin ella.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantilla/Agenda-semanal-hoja.xlsx
+++ b/plantilla/Agenda-semanal-hoja.xlsx
@@ -606,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H403"/>
+  <dimension ref="A1:I403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -617,6 +617,7 @@
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -629,7 +630,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Una fila por evento. Rellena Fecha, Categoría y Título (Hora, Texto y Enlace son opcionales). Hora: 9:00 o 9:00-14:00. Día y Semana (de domingo a sábado) se calculan solos. El orden da igual: la web lo coloca en su día.</t>
+          <t>Una fila por evento. Rellena Fecha, Categoría y Título (Hora, Texto, Enlace y Foto son opcionales). Hora: 9:00 o 9:00-14:00. Día y Semana (de domingo a sábado) se calculan solos. El orden da igual: la web lo coloca en su día.</t>
         </is>
       </c>
     </row>
@@ -674,6 +675,11 @@
           <t>Enlace</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="n">
@@ -708,6 +714,7 @@
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr"/>
+      <c r="I4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="n">
@@ -738,6 +745,7 @@
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n">
@@ -768,6 +776,7 @@
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
+      <c r="I6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
@@ -798,6 +807,7 @@
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
@@ -832,6 +842,7 @@
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
@@ -866,6 +877,7 @@
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="n">
@@ -900,6 +912,7 @@
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n">
@@ -930,6 +943,7 @@
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
@@ -960,6 +974,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr"/>
       <c r="H12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="n">
@@ -994,6 +1009,7 @@
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="n">
@@ -1028,6 +1044,7 @@
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="n"/>
@@ -1044,6 +1061,7 @@
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="n"/>
@@ -1060,6 +1078,7 @@
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="n"/>
@@ -1076,6 +1095,7 @@
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="7" t="n"/>
       <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="n"/>
@@ -1092,6 +1112,7 @@
       <c r="F18" s="8" t="n"/>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="n"/>
@@ -1108,6 +1129,7 @@
       <c r="F19" s="8" t="n"/>
       <c r="G19" s="7" t="n"/>
       <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="n"/>
@@ -1124,6 +1146,7 @@
       <c r="F20" s="8" t="n"/>
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="n"/>
@@ -1140,6 +1163,7 @@
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="n"/>
@@ -1156,6 +1180,7 @@
       <c r="F22" s="8" t="n"/>
       <c r="G22" s="7" t="n"/>
       <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="12" t="n"/>
@@ -1172,6 +1197,7 @@
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="7" t="n"/>
       <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="n"/>
@@ -1188,6 +1214,7 @@
       <c r="F24" s="8" t="n"/>
       <c r="G24" s="7" t="n"/>
       <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="n"/>
@@ -1204,6 +1231,7 @@
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="n"/>
@@ -1220,6 +1248,7 @@
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="7" t="n"/>
       <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n"/>
@@ -1236,6 +1265,7 @@
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n"/>
@@ -1252,6 +1282,7 @@
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="7" t="n"/>
       <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n"/>
@@ -1268,6 +1299,7 @@
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="n"/>
@@ -1284,6 +1316,7 @@
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="7" t="n"/>
       <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="n"/>
@@ -1300,6 +1333,7 @@
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="7" t="n"/>
       <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n"/>
@@ -1316,6 +1350,7 @@
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="7" t="n"/>
       <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12" t="n"/>
@@ -1332,6 +1367,7 @@
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="7" t="n"/>
       <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="12" t="n"/>
@@ -1348,6 +1384,7 @@
       <c r="F34" s="8" t="n"/>
       <c r="G34" s="7" t="n"/>
       <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="12" t="n"/>
@@ -1364,6 +1401,7 @@
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="n"/>
@@ -1380,6 +1418,7 @@
       <c r="F36" s="8" t="n"/>
       <c r="G36" s="7" t="n"/>
       <c r="H36" s="7" t="n"/>
+      <c r="I36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n"/>
@@ -1396,6 +1435,7 @@
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="7" t="n"/>
       <c r="H37" s="7" t="n"/>
+      <c r="I37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="12" t="n"/>
@@ -1412,6 +1452,7 @@
       <c r="F38" s="8" t="n"/>
       <c r="G38" s="7" t="n"/>
       <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="12" t="n"/>
@@ -1428,6 +1469,7 @@
       <c r="F39" s="8" t="n"/>
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="n"/>
@@ -1444,6 +1486,7 @@
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="7" t="n"/>
       <c r="H40" s="7" t="n"/>
+      <c r="I40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n"/>
@@ -1460,6 +1503,7 @@
       <c r="F41" s="8" t="n"/>
       <c r="G41" s="7" t="n"/>
       <c r="H41" s="7" t="n"/>
+      <c r="I41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="n"/>
@@ -1476,6 +1520,7 @@
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="7" t="n"/>
       <c r="H42" s="7" t="n"/>
+      <c r="I42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="12" t="n"/>
@@ -1492,6 +1537,7 @@
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="7" t="n"/>
       <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="12" t="n"/>
@@ -1508,6 +1554,7 @@
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="7" t="n"/>
       <c r="H44" s="7" t="n"/>
+      <c r="I44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="12" t="n"/>
@@ -1524,6 +1571,7 @@
       <c r="F45" s="8" t="n"/>
       <c r="G45" s="7" t="n"/>
       <c r="H45" s="7" t="n"/>
+      <c r="I45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="12" t="n"/>
@@ -1540,6 +1588,7 @@
       <c r="F46" s="8" t="n"/>
       <c r="G46" s="7" t="n"/>
       <c r="H46" s="7" t="n"/>
+      <c r="I46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="12" t="n"/>
@@ -1556,6 +1605,7 @@
       <c r="F47" s="8" t="n"/>
       <c r="G47" s="7" t="n"/>
       <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="12" t="n"/>
@@ -1572,6 +1622,7 @@
       <c r="F48" s="8" t="n"/>
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="12" t="n"/>
@@ -1588,6 +1639,7 @@
       <c r="F49" s="8" t="n"/>
       <c r="G49" s="7" t="n"/>
       <c r="H49" s="7" t="n"/>
+      <c r="I49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="12" t="n"/>
@@ -1604,6 +1656,7 @@
       <c r="F50" s="8" t="n"/>
       <c r="G50" s="7" t="n"/>
       <c r="H50" s="7" t="n"/>
+      <c r="I50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="12" t="n"/>
@@ -1620,6 +1673,7 @@
       <c r="F51" s="8" t="n"/>
       <c r="G51" s="7" t="n"/>
       <c r="H51" s="7" t="n"/>
+      <c r="I51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="12" t="n"/>
@@ -1636,6 +1690,7 @@
       <c r="F52" s="8" t="n"/>
       <c r="G52" s="7" t="n"/>
       <c r="H52" s="7" t="n"/>
+      <c r="I52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="12" t="n"/>
@@ -1652,6 +1707,7 @@
       <c r="F53" s="8" t="n"/>
       <c r="G53" s="7" t="n"/>
       <c r="H53" s="7" t="n"/>
+      <c r="I53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="12" t="n"/>
@@ -1668,6 +1724,7 @@
       <c r="F54" s="8" t="n"/>
       <c r="G54" s="7" t="n"/>
       <c r="H54" s="7" t="n"/>
+      <c r="I54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="12" t="n"/>
@@ -1684,6 +1741,7 @@
       <c r="F55" s="8" t="n"/>
       <c r="G55" s="7" t="n"/>
       <c r="H55" s="7" t="n"/>
+      <c r="I55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="12" t="n"/>
@@ -1700,6 +1758,7 @@
       <c r="F56" s="8" t="n"/>
       <c r="G56" s="7" t="n"/>
       <c r="H56" s="7" t="n"/>
+      <c r="I56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="12" t="n"/>
@@ -1716,6 +1775,7 @@
       <c r="F57" s="8" t="n"/>
       <c r="G57" s="7" t="n"/>
       <c r="H57" s="7" t="n"/>
+      <c r="I57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="12" t="n"/>
@@ -1732,6 +1792,7 @@
       <c r="F58" s="8" t="n"/>
       <c r="G58" s="7" t="n"/>
       <c r="H58" s="7" t="n"/>
+      <c r="I58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="12" t="n"/>
@@ -1748,6 +1809,7 @@
       <c r="F59" s="8" t="n"/>
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
+      <c r="I59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="n"/>
@@ -1764,6 +1826,7 @@
       <c r="F60" s="8" t="n"/>
       <c r="G60" s="7" t="n"/>
       <c r="H60" s="7" t="n"/>
+      <c r="I60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n"/>
@@ -1780,6 +1843,7 @@
       <c r="F61" s="8" t="n"/>
       <c r="G61" s="7" t="n"/>
       <c r="H61" s="7" t="n"/>
+      <c r="I61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="n"/>
@@ -1796,6 +1860,7 @@
       <c r="F62" s="8" t="n"/>
       <c r="G62" s="7" t="n"/>
       <c r="H62" s="7" t="n"/>
+      <c r="I62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="12" t="n"/>
@@ -1812,6 +1877,7 @@
       <c r="F63" s="8" t="n"/>
       <c r="G63" s="7" t="n"/>
       <c r="H63" s="7" t="n"/>
+      <c r="I63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="n"/>
@@ -1828,6 +1894,7 @@
       <c r="F64" s="8" t="n"/>
       <c r="G64" s="7" t="n"/>
       <c r="H64" s="7" t="n"/>
+      <c r="I64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="12" t="n"/>
@@ -1844,6 +1911,7 @@
       <c r="F65" s="8" t="n"/>
       <c r="G65" s="7" t="n"/>
       <c r="H65" s="7" t="n"/>
+      <c r="I65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="n"/>
@@ -1860,6 +1928,7 @@
       <c r="F66" s="8" t="n"/>
       <c r="G66" s="7" t="n"/>
       <c r="H66" s="7" t="n"/>
+      <c r="I66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="n"/>
@@ -1876,6 +1945,7 @@
       <c r="F67" s="8" t="n"/>
       <c r="G67" s="7" t="n"/>
       <c r="H67" s="7" t="n"/>
+      <c r="I67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="12" t="n"/>
@@ -1892,6 +1962,7 @@
       <c r="F68" s="8" t="n"/>
       <c r="G68" s="7" t="n"/>
       <c r="H68" s="7" t="n"/>
+      <c r="I68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="12" t="n"/>
@@ -1908,6 +1979,7 @@
       <c r="F69" s="8" t="n"/>
       <c r="G69" s="7" t="n"/>
       <c r="H69" s="7" t="n"/>
+      <c r="I69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="12" t="n"/>
@@ -1924,6 +1996,7 @@
       <c r="F70" s="8" t="n"/>
       <c r="G70" s="7" t="n"/>
       <c r="H70" s="7" t="n"/>
+      <c r="I70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="12" t="n"/>
@@ -1940,6 +2013,7 @@
       <c r="F71" s="8" t="n"/>
       <c r="G71" s="7" t="n"/>
       <c r="H71" s="7" t="n"/>
+      <c r="I71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="12" t="n"/>
@@ -1956,6 +2030,7 @@
       <c r="F72" s="8" t="n"/>
       <c r="G72" s="7" t="n"/>
       <c r="H72" s="7" t="n"/>
+      <c r="I72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="12" t="n"/>
@@ -1972,6 +2047,7 @@
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="7" t="n"/>
       <c r="H73" s="7" t="n"/>
+      <c r="I73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="12" t="n"/>
@@ -1988,6 +2064,7 @@
       <c r="F74" s="8" t="n"/>
       <c r="G74" s="7" t="n"/>
       <c r="H74" s="7" t="n"/>
+      <c r="I74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="12" t="n"/>
@@ -2004,6 +2081,7 @@
       <c r="F75" s="8" t="n"/>
       <c r="G75" s="7" t="n"/>
       <c r="H75" s="7" t="n"/>
+      <c r="I75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="12" t="n"/>
@@ -2020,6 +2098,7 @@
       <c r="F76" s="8" t="n"/>
       <c r="G76" s="7" t="n"/>
       <c r="H76" s="7" t="n"/>
+      <c r="I76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="12" t="n"/>
@@ -2036,6 +2115,7 @@
       <c r="F77" s="8" t="n"/>
       <c r="G77" s="7" t="n"/>
       <c r="H77" s="7" t="n"/>
+      <c r="I77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="12" t="n"/>
@@ -2052,6 +2132,7 @@
       <c r="F78" s="8" t="n"/>
       <c r="G78" s="7" t="n"/>
       <c r="H78" s="7" t="n"/>
+      <c r="I78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="12" t="n"/>
@@ -2068,6 +2149,7 @@
       <c r="F79" s="8" t="n"/>
       <c r="G79" s="7" t="n"/>
       <c r="H79" s="7" t="n"/>
+      <c r="I79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="12" t="n"/>
@@ -2084,6 +2166,7 @@
       <c r="F80" s="8" t="n"/>
       <c r="G80" s="7" t="n"/>
       <c r="H80" s="7" t="n"/>
+      <c r="I80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="12" t="n"/>
@@ -2100,6 +2183,7 @@
       <c r="F81" s="8" t="n"/>
       <c r="G81" s="7" t="n"/>
       <c r="H81" s="7" t="n"/>
+      <c r="I81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="12" t="n"/>
@@ -2116,6 +2200,7 @@
       <c r="F82" s="8" t="n"/>
       <c r="G82" s="7" t="n"/>
       <c r="H82" s="7" t="n"/>
+      <c r="I82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="12" t="n"/>
@@ -2132,6 +2217,7 @@
       <c r="F83" s="8" t="n"/>
       <c r="G83" s="7" t="n"/>
       <c r="H83" s="7" t="n"/>
+      <c r="I83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="12" t="n"/>
@@ -2148,6 +2234,7 @@
       <c r="F84" s="8" t="n"/>
       <c r="G84" s="7" t="n"/>
       <c r="H84" s="7" t="n"/>
+      <c r="I84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="12" t="n"/>
@@ -2164,6 +2251,7 @@
       <c r="F85" s="8" t="n"/>
       <c r="G85" s="7" t="n"/>
       <c r="H85" s="7" t="n"/>
+      <c r="I85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="12" t="n"/>
@@ -2180,6 +2268,7 @@
       <c r="F86" s="8" t="n"/>
       <c r="G86" s="7" t="n"/>
       <c r="H86" s="7" t="n"/>
+      <c r="I86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="12" t="n"/>
@@ -2196,6 +2285,7 @@
       <c r="F87" s="8" t="n"/>
       <c r="G87" s="7" t="n"/>
       <c r="H87" s="7" t="n"/>
+      <c r="I87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="12" t="n"/>
@@ -2212,6 +2302,7 @@
       <c r="F88" s="8" t="n"/>
       <c r="G88" s="7" t="n"/>
       <c r="H88" s="7" t="n"/>
+      <c r="I88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="12" t="n"/>
@@ -2228,6 +2319,7 @@
       <c r="F89" s="8" t="n"/>
       <c r="G89" s="7" t="n"/>
       <c r="H89" s="7" t="n"/>
+      <c r="I89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="12" t="n"/>
@@ -2244,6 +2336,7 @@
       <c r="F90" s="8" t="n"/>
       <c r="G90" s="7" t="n"/>
       <c r="H90" s="7" t="n"/>
+      <c r="I90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="12" t="n"/>
@@ -2260,6 +2353,7 @@
       <c r="F91" s="8" t="n"/>
       <c r="G91" s="7" t="n"/>
       <c r="H91" s="7" t="n"/>
+      <c r="I91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="12" t="n"/>
@@ -2276,6 +2370,7 @@
       <c r="F92" s="8" t="n"/>
       <c r="G92" s="7" t="n"/>
       <c r="H92" s="7" t="n"/>
+      <c r="I92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="12" t="n"/>
@@ -2292,6 +2387,7 @@
       <c r="F93" s="8" t="n"/>
       <c r="G93" s="7" t="n"/>
       <c r="H93" s="7" t="n"/>
+      <c r="I93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="12" t="n"/>
@@ -2308,6 +2404,7 @@
       <c r="F94" s="8" t="n"/>
       <c r="G94" s="7" t="n"/>
       <c r="H94" s="7" t="n"/>
+      <c r="I94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="12" t="n"/>
@@ -2324,6 +2421,7 @@
       <c r="F95" s="8" t="n"/>
       <c r="G95" s="7" t="n"/>
       <c r="H95" s="7" t="n"/>
+      <c r="I95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="12" t="n"/>
@@ -2340,6 +2438,7 @@
       <c r="F96" s="8" t="n"/>
       <c r="G96" s="7" t="n"/>
       <c r="H96" s="7" t="n"/>
+      <c r="I96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="12" t="n"/>
@@ -2356,6 +2455,7 @@
       <c r="F97" s="8" t="n"/>
       <c r="G97" s="7" t="n"/>
       <c r="H97" s="7" t="n"/>
+      <c r="I97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="12" t="n"/>
@@ -2372,6 +2472,7 @@
       <c r="F98" s="8" t="n"/>
       <c r="G98" s="7" t="n"/>
       <c r="H98" s="7" t="n"/>
+      <c r="I98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="12" t="n"/>
@@ -2388,6 +2489,7 @@
       <c r="F99" s="8" t="n"/>
       <c r="G99" s="7" t="n"/>
       <c r="H99" s="7" t="n"/>
+      <c r="I99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="12" t="n"/>
@@ -2404,6 +2506,7 @@
       <c r="F100" s="8" t="n"/>
       <c r="G100" s="7" t="n"/>
       <c r="H100" s="7" t="n"/>
+      <c r="I100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="12" t="n"/>
@@ -2420,6 +2523,7 @@
       <c r="F101" s="8" t="n"/>
       <c r="G101" s="7" t="n"/>
       <c r="H101" s="7" t="n"/>
+      <c r="I101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="12" t="n"/>
@@ -2436,6 +2540,7 @@
       <c r="F102" s="8" t="n"/>
       <c r="G102" s="7" t="n"/>
       <c r="H102" s="7" t="n"/>
+      <c r="I102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="12" t="n"/>
@@ -2452,6 +2557,7 @@
       <c r="F103" s="8" t="n"/>
       <c r="G103" s="7" t="n"/>
       <c r="H103" s="7" t="n"/>
+      <c r="I103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="12" t="n"/>
@@ -2468,6 +2574,7 @@
       <c r="F104" s="8" t="n"/>
       <c r="G104" s="7" t="n"/>
       <c r="H104" s="7" t="n"/>
+      <c r="I104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="12" t="n"/>
@@ -2484,6 +2591,7 @@
       <c r="F105" s="8" t="n"/>
       <c r="G105" s="7" t="n"/>
       <c r="H105" s="7" t="n"/>
+      <c r="I105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="12" t="n"/>
@@ -2500,6 +2608,7 @@
       <c r="F106" s="8" t="n"/>
       <c r="G106" s="7" t="n"/>
       <c r="H106" s="7" t="n"/>
+      <c r="I106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="12" t="n"/>
@@ -2516,6 +2625,7 @@
       <c r="F107" s="8" t="n"/>
       <c r="G107" s="7" t="n"/>
       <c r="H107" s="7" t="n"/>
+      <c r="I107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="12" t="n"/>
@@ -2532,6 +2642,7 @@
       <c r="F108" s="8" t="n"/>
       <c r="G108" s="7" t="n"/>
       <c r="H108" s="7" t="n"/>
+      <c r="I108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="12" t="n"/>
@@ -2548,6 +2659,7 @@
       <c r="F109" s="8" t="n"/>
       <c r="G109" s="7" t="n"/>
       <c r="H109" s="7" t="n"/>
+      <c r="I109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="12" t="n"/>
@@ -2564,6 +2676,7 @@
       <c r="F110" s="8" t="n"/>
       <c r="G110" s="7" t="n"/>
       <c r="H110" s="7" t="n"/>
+      <c r="I110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="12" t="n"/>
@@ -2580,6 +2693,7 @@
       <c r="F111" s="8" t="n"/>
       <c r="G111" s="7" t="n"/>
       <c r="H111" s="7" t="n"/>
+      <c r="I111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="12" t="n"/>
@@ -2596,6 +2710,7 @@
       <c r="F112" s="8" t="n"/>
       <c r="G112" s="7" t="n"/>
       <c r="H112" s="7" t="n"/>
+      <c r="I112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="12" t="n"/>
@@ -2612,6 +2727,7 @@
       <c r="F113" s="8" t="n"/>
       <c r="G113" s="7" t="n"/>
       <c r="H113" s="7" t="n"/>
+      <c r="I113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="12" t="n"/>
@@ -2628,6 +2744,7 @@
       <c r="F114" s="8" t="n"/>
       <c r="G114" s="7" t="n"/>
       <c r="H114" s="7" t="n"/>
+      <c r="I114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="12" t="n"/>
@@ -2644,6 +2761,7 @@
       <c r="F115" s="8" t="n"/>
       <c r="G115" s="7" t="n"/>
       <c r="H115" s="7" t="n"/>
+      <c r="I115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="12" t="n"/>
@@ -2660,6 +2778,7 @@
       <c r="F116" s="8" t="n"/>
       <c r="G116" s="7" t="n"/>
       <c r="H116" s="7" t="n"/>
+      <c r="I116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="12" t="n"/>
@@ -2676,6 +2795,7 @@
       <c r="F117" s="8" t="n"/>
       <c r="G117" s="7" t="n"/>
       <c r="H117" s="7" t="n"/>
+      <c r="I117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="12" t="n"/>
@@ -2692,6 +2812,7 @@
       <c r="F118" s="8" t="n"/>
       <c r="G118" s="7" t="n"/>
       <c r="H118" s="7" t="n"/>
+      <c r="I118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="12" t="n"/>
@@ -2708,6 +2829,7 @@
       <c r="F119" s="8" t="n"/>
       <c r="G119" s="7" t="n"/>
       <c r="H119" s="7" t="n"/>
+      <c r="I119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="12" t="n"/>
@@ -2724,6 +2846,7 @@
       <c r="F120" s="8" t="n"/>
       <c r="G120" s="7" t="n"/>
       <c r="H120" s="7" t="n"/>
+      <c r="I120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="12" t="n"/>
@@ -2740,6 +2863,7 @@
       <c r="F121" s="8" t="n"/>
       <c r="G121" s="7" t="n"/>
       <c r="H121" s="7" t="n"/>
+      <c r="I121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="12" t="n"/>
@@ -2756,6 +2880,7 @@
       <c r="F122" s="8" t="n"/>
       <c r="G122" s="7" t="n"/>
       <c r="H122" s="7" t="n"/>
+      <c r="I122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="12" t="n"/>
@@ -2772,6 +2897,7 @@
       <c r="F123" s="8" t="n"/>
       <c r="G123" s="7" t="n"/>
       <c r="H123" s="7" t="n"/>
+      <c r="I123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="12" t="n"/>
@@ -2788,6 +2914,7 @@
       <c r="F124" s="8" t="n"/>
       <c r="G124" s="7" t="n"/>
       <c r="H124" s="7" t="n"/>
+      <c r="I124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="12" t="n"/>
@@ -2804,6 +2931,7 @@
       <c r="F125" s="8" t="n"/>
       <c r="G125" s="7" t="n"/>
       <c r="H125" s="7" t="n"/>
+      <c r="I125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="12" t="n"/>
@@ -2820,6 +2948,7 @@
       <c r="F126" s="8" t="n"/>
       <c r="G126" s="7" t="n"/>
       <c r="H126" s="7" t="n"/>
+      <c r="I126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="12" t="n"/>
@@ -2836,6 +2965,7 @@
       <c r="F127" s="8" t="n"/>
       <c r="G127" s="7" t="n"/>
       <c r="H127" s="7" t="n"/>
+      <c r="I127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="12" t="n"/>
@@ -2852,6 +2982,7 @@
       <c r="F128" s="8" t="n"/>
       <c r="G128" s="7" t="n"/>
       <c r="H128" s="7" t="n"/>
+      <c r="I128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="12" t="n"/>
@@ -2868,6 +2999,7 @@
       <c r="F129" s="8" t="n"/>
       <c r="G129" s="7" t="n"/>
       <c r="H129" s="7" t="n"/>
+      <c r="I129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="12" t="n"/>
@@ -2884,6 +3016,7 @@
       <c r="F130" s="8" t="n"/>
       <c r="G130" s="7" t="n"/>
       <c r="H130" s="7" t="n"/>
+      <c r="I130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="12" t="n"/>
@@ -2900,6 +3033,7 @@
       <c r="F131" s="8" t="n"/>
       <c r="G131" s="7" t="n"/>
       <c r="H131" s="7" t="n"/>
+      <c r="I131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="12" t="n"/>
@@ -2916,6 +3050,7 @@
       <c r="F132" s="8" t="n"/>
       <c r="G132" s="7" t="n"/>
       <c r="H132" s="7" t="n"/>
+      <c r="I132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="12" t="n"/>
@@ -2932,6 +3067,7 @@
       <c r="F133" s="8" t="n"/>
       <c r="G133" s="7" t="n"/>
       <c r="H133" s="7" t="n"/>
+      <c r="I133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="12" t="n"/>
@@ -2948,6 +3084,7 @@
       <c r="F134" s="8" t="n"/>
       <c r="G134" s="7" t="n"/>
       <c r="H134" s="7" t="n"/>
+      <c r="I134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="12" t="n"/>
@@ -2964,6 +3101,7 @@
       <c r="F135" s="8" t="n"/>
       <c r="G135" s="7" t="n"/>
       <c r="H135" s="7" t="n"/>
+      <c r="I135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="12" t="n"/>
@@ -2980,6 +3118,7 @@
       <c r="F136" s="8" t="n"/>
       <c r="G136" s="7" t="n"/>
       <c r="H136" s="7" t="n"/>
+      <c r="I136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="12" t="n"/>
@@ -2996,6 +3135,7 @@
       <c r="F137" s="8" t="n"/>
       <c r="G137" s="7" t="n"/>
       <c r="H137" s="7" t="n"/>
+      <c r="I137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="12" t="n"/>
@@ -3012,6 +3152,7 @@
       <c r="F138" s="8" t="n"/>
       <c r="G138" s="7" t="n"/>
       <c r="H138" s="7" t="n"/>
+      <c r="I138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="12" t="n"/>
@@ -3028,6 +3169,7 @@
       <c r="F139" s="8" t="n"/>
       <c r="G139" s="7" t="n"/>
       <c r="H139" s="7" t="n"/>
+      <c r="I139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="12" t="n"/>
@@ -3044,6 +3186,7 @@
       <c r="F140" s="8" t="n"/>
       <c r="G140" s="7" t="n"/>
       <c r="H140" s="7" t="n"/>
+      <c r="I140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="12" t="n"/>
@@ -3060,6 +3203,7 @@
       <c r="F141" s="8" t="n"/>
       <c r="G141" s="7" t="n"/>
       <c r="H141" s="7" t="n"/>
+      <c r="I141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="12" t="n"/>
@@ -3076,6 +3220,7 @@
       <c r="F142" s="8" t="n"/>
       <c r="G142" s="7" t="n"/>
       <c r="H142" s="7" t="n"/>
+      <c r="I142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="12" t="n"/>
@@ -3092,6 +3237,7 @@
       <c r="F143" s="8" t="n"/>
       <c r="G143" s="7" t="n"/>
       <c r="H143" s="7" t="n"/>
+      <c r="I143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="12" t="n"/>
@@ -3108,6 +3254,7 @@
       <c r="F144" s="8" t="n"/>
       <c r="G144" s="7" t="n"/>
       <c r="H144" s="7" t="n"/>
+      <c r="I144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="12" t="n"/>
@@ -3124,6 +3271,7 @@
       <c r="F145" s="8" t="n"/>
       <c r="G145" s="7" t="n"/>
       <c r="H145" s="7" t="n"/>
+      <c r="I145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="12" t="n"/>
@@ -3140,6 +3288,7 @@
       <c r="F146" s="8" t="n"/>
       <c r="G146" s="7" t="n"/>
       <c r="H146" s="7" t="n"/>
+      <c r="I146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="12" t="n"/>
@@ -3156,6 +3305,7 @@
       <c r="F147" s="8" t="n"/>
       <c r="G147" s="7" t="n"/>
       <c r="H147" s="7" t="n"/>
+      <c r="I147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="12" t="n"/>
@@ -3172,6 +3322,7 @@
       <c r="F148" s="8" t="n"/>
       <c r="G148" s="7" t="n"/>
       <c r="H148" s="7" t="n"/>
+      <c r="I148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="12" t="n"/>
@@ -3188,6 +3339,7 @@
       <c r="F149" s="8" t="n"/>
       <c r="G149" s="7" t="n"/>
       <c r="H149" s="7" t="n"/>
+      <c r="I149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="12" t="n"/>
@@ -3204,6 +3356,7 @@
       <c r="F150" s="8" t="n"/>
       <c r="G150" s="7" t="n"/>
       <c r="H150" s="7" t="n"/>
+      <c r="I150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="12" t="n"/>
@@ -3220,6 +3373,7 @@
       <c r="F151" s="8" t="n"/>
       <c r="G151" s="7" t="n"/>
       <c r="H151" s="7" t="n"/>
+      <c r="I151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="12" t="n"/>
@@ -3236,6 +3390,7 @@
       <c r="F152" s="8" t="n"/>
       <c r="G152" s="7" t="n"/>
       <c r="H152" s="7" t="n"/>
+      <c r="I152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="12" t="n"/>
@@ -3252,6 +3407,7 @@
       <c r="F153" s="8" t="n"/>
       <c r="G153" s="7" t="n"/>
       <c r="H153" s="7" t="n"/>
+      <c r="I153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="12" t="n"/>
@@ -3268,6 +3424,7 @@
       <c r="F154" s="8" t="n"/>
       <c r="G154" s="7" t="n"/>
       <c r="H154" s="7" t="n"/>
+      <c r="I154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="12" t="n"/>
@@ -3284,6 +3441,7 @@
       <c r="F155" s="8" t="n"/>
       <c r="G155" s="7" t="n"/>
       <c r="H155" s="7" t="n"/>
+      <c r="I155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="12" t="n"/>
@@ -3300,6 +3458,7 @@
       <c r="F156" s="8" t="n"/>
       <c r="G156" s="7" t="n"/>
       <c r="H156" s="7" t="n"/>
+      <c r="I156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="12" t="n"/>
@@ -3316,6 +3475,7 @@
       <c r="F157" s="8" t="n"/>
       <c r="G157" s="7" t="n"/>
       <c r="H157" s="7" t="n"/>
+      <c r="I157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="12" t="n"/>
@@ -3332,6 +3492,7 @@
       <c r="F158" s="8" t="n"/>
       <c r="G158" s="7" t="n"/>
       <c r="H158" s="7" t="n"/>
+      <c r="I158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="12" t="n"/>
@@ -3348,6 +3509,7 @@
       <c r="F159" s="8" t="n"/>
       <c r="G159" s="7" t="n"/>
       <c r="H159" s="7" t="n"/>
+      <c r="I159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="12" t="n"/>
@@ -3364,6 +3526,7 @@
       <c r="F160" s="8" t="n"/>
       <c r="G160" s="7" t="n"/>
       <c r="H160" s="7" t="n"/>
+      <c r="I160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="12" t="n"/>
@@ -3380,6 +3543,7 @@
       <c r="F161" s="8" t="n"/>
       <c r="G161" s="7" t="n"/>
       <c r="H161" s="7" t="n"/>
+      <c r="I161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="12" t="n"/>
@@ -3396,6 +3560,7 @@
       <c r="F162" s="8" t="n"/>
       <c r="G162" s="7" t="n"/>
       <c r="H162" s="7" t="n"/>
+      <c r="I162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="12" t="n"/>
@@ -3412,6 +3577,7 @@
       <c r="F163" s="8" t="n"/>
       <c r="G163" s="7" t="n"/>
       <c r="H163" s="7" t="n"/>
+      <c r="I163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="12" t="n"/>
@@ -3428,6 +3594,7 @@
       <c r="F164" s="8" t="n"/>
       <c r="G164" s="7" t="n"/>
       <c r="H164" s="7" t="n"/>
+      <c r="I164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="12" t="n"/>
@@ -3444,6 +3611,7 @@
       <c r="F165" s="8" t="n"/>
       <c r="G165" s="7" t="n"/>
       <c r="H165" s="7" t="n"/>
+      <c r="I165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="12" t="n"/>
@@ -3460,6 +3628,7 @@
       <c r="F166" s="8" t="n"/>
       <c r="G166" s="7" t="n"/>
       <c r="H166" s="7" t="n"/>
+      <c r="I166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="12" t="n"/>
@@ -3476,6 +3645,7 @@
       <c r="F167" s="8" t="n"/>
       <c r="G167" s="7" t="n"/>
       <c r="H167" s="7" t="n"/>
+      <c r="I167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="12" t="n"/>
@@ -3492,6 +3662,7 @@
       <c r="F168" s="8" t="n"/>
       <c r="G168" s="7" t="n"/>
       <c r="H168" s="7" t="n"/>
+      <c r="I168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="12" t="n"/>
@@ -3508,6 +3679,7 @@
       <c r="F169" s="8" t="n"/>
       <c r="G169" s="7" t="n"/>
       <c r="H169" s="7" t="n"/>
+      <c r="I169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="12" t="n"/>
@@ -3524,6 +3696,7 @@
       <c r="F170" s="8" t="n"/>
       <c r="G170" s="7" t="n"/>
       <c r="H170" s="7" t="n"/>
+      <c r="I170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="12" t="n"/>
@@ -3540,6 +3713,7 @@
       <c r="F171" s="8" t="n"/>
       <c r="G171" s="7" t="n"/>
       <c r="H171" s="7" t="n"/>
+      <c r="I171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="12" t="n"/>
@@ -3556,6 +3730,7 @@
       <c r="F172" s="8" t="n"/>
       <c r="G172" s="7" t="n"/>
       <c r="H172" s="7" t="n"/>
+      <c r="I172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="12" t="n"/>
@@ -3572,6 +3747,7 @@
       <c r="F173" s="8" t="n"/>
       <c r="G173" s="7" t="n"/>
       <c r="H173" s="7" t="n"/>
+      <c r="I173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="12" t="n"/>
@@ -3588,6 +3764,7 @@
       <c r="F174" s="8" t="n"/>
       <c r="G174" s="7" t="n"/>
       <c r="H174" s="7" t="n"/>
+      <c r="I174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="12" t="n"/>
@@ -3604,6 +3781,7 @@
       <c r="F175" s="8" t="n"/>
       <c r="G175" s="7" t="n"/>
       <c r="H175" s="7" t="n"/>
+      <c r="I175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="12" t="n"/>
@@ -3620,6 +3798,7 @@
       <c r="F176" s="8" t="n"/>
       <c r="G176" s="7" t="n"/>
       <c r="H176" s="7" t="n"/>
+      <c r="I176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="12" t="n"/>
@@ -3636,6 +3815,7 @@
       <c r="F177" s="8" t="n"/>
       <c r="G177" s="7" t="n"/>
       <c r="H177" s="7" t="n"/>
+      <c r="I177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="12" t="n"/>
@@ -3652,6 +3832,7 @@
       <c r="F178" s="8" t="n"/>
       <c r="G178" s="7" t="n"/>
       <c r="H178" s="7" t="n"/>
+      <c r="I178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="12" t="n"/>
@@ -3668,6 +3849,7 @@
       <c r="F179" s="8" t="n"/>
       <c r="G179" s="7" t="n"/>
       <c r="H179" s="7" t="n"/>
+      <c r="I179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="12" t="n"/>
@@ -3684,6 +3866,7 @@
       <c r="F180" s="8" t="n"/>
       <c r="G180" s="7" t="n"/>
       <c r="H180" s="7" t="n"/>
+      <c r="I180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="12" t="n"/>
@@ -3700,6 +3883,7 @@
       <c r="F181" s="8" t="n"/>
       <c r="G181" s="7" t="n"/>
       <c r="H181" s="7" t="n"/>
+      <c r="I181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="12" t="n"/>
@@ -3716,6 +3900,7 @@
       <c r="F182" s="8" t="n"/>
       <c r="G182" s="7" t="n"/>
       <c r="H182" s="7" t="n"/>
+      <c r="I182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="12" t="n"/>
@@ -3732,6 +3917,7 @@
       <c r="F183" s="8" t="n"/>
       <c r="G183" s="7" t="n"/>
       <c r="H183" s="7" t="n"/>
+      <c r="I183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="12" t="n"/>
@@ -3748,6 +3934,7 @@
       <c r="F184" s="8" t="n"/>
       <c r="G184" s="7" t="n"/>
       <c r="H184" s="7" t="n"/>
+      <c r="I184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="12" t="n"/>
@@ -3764,6 +3951,7 @@
       <c r="F185" s="8" t="n"/>
       <c r="G185" s="7" t="n"/>
       <c r="H185" s="7" t="n"/>
+      <c r="I185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="12" t="n"/>
@@ -3780,6 +3968,7 @@
       <c r="F186" s="8" t="n"/>
       <c r="G186" s="7" t="n"/>
       <c r="H186" s="7" t="n"/>
+      <c r="I186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="12" t="n"/>
@@ -3796,6 +3985,7 @@
       <c r="F187" s="8" t="n"/>
       <c r="G187" s="7" t="n"/>
       <c r="H187" s="7" t="n"/>
+      <c r="I187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="12" t="n"/>
@@ -3812,6 +4002,7 @@
       <c r="F188" s="8" t="n"/>
       <c r="G188" s="7" t="n"/>
       <c r="H188" s="7" t="n"/>
+      <c r="I188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="12" t="n"/>
@@ -3828,6 +4019,7 @@
       <c r="F189" s="8" t="n"/>
       <c r="G189" s="7" t="n"/>
       <c r="H189" s="7" t="n"/>
+      <c r="I189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="12" t="n"/>
@@ -3844,6 +4036,7 @@
       <c r="F190" s="8" t="n"/>
       <c r="G190" s="7" t="n"/>
       <c r="H190" s="7" t="n"/>
+      <c r="I190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="12" t="n"/>
@@ -3860,6 +4053,7 @@
       <c r="F191" s="8" t="n"/>
       <c r="G191" s="7" t="n"/>
       <c r="H191" s="7" t="n"/>
+      <c r="I191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="12" t="n"/>
@@ -3876,6 +4070,7 @@
       <c r="F192" s="8" t="n"/>
       <c r="G192" s="7" t="n"/>
       <c r="H192" s="7" t="n"/>
+      <c r="I192" s="7" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="12" t="n"/>
@@ -3892,6 +4087,7 @@
       <c r="F193" s="8" t="n"/>
       <c r="G193" s="7" t="n"/>
       <c r="H193" s="7" t="n"/>
+      <c r="I193" s="7" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="12" t="n"/>
@@ -3908,6 +4104,7 @@
       <c r="F194" s="8" t="n"/>
       <c r="G194" s="7" t="n"/>
       <c r="H194" s="7" t="n"/>
+      <c r="I194" s="7" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="12" t="n"/>
@@ -3924,6 +4121,7 @@
       <c r="F195" s="8" t="n"/>
       <c r="G195" s="7" t="n"/>
       <c r="H195" s="7" t="n"/>
+      <c r="I195" s="7" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="12" t="n"/>
@@ -3940,6 +4138,7 @@
       <c r="F196" s="8" t="n"/>
       <c r="G196" s="7" t="n"/>
       <c r="H196" s="7" t="n"/>
+      <c r="I196" s="7" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="12" t="n"/>
@@ -3956,6 +4155,7 @@
       <c r="F197" s="8" t="n"/>
       <c r="G197" s="7" t="n"/>
       <c r="H197" s="7" t="n"/>
+      <c r="I197" s="7" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="12" t="n"/>
@@ -3972,6 +4172,7 @@
       <c r="F198" s="8" t="n"/>
       <c r="G198" s="7" t="n"/>
       <c r="H198" s="7" t="n"/>
+      <c r="I198" s="7" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="12" t="n"/>
@@ -3988,6 +4189,7 @@
       <c r="F199" s="8" t="n"/>
       <c r="G199" s="7" t="n"/>
       <c r="H199" s="7" t="n"/>
+      <c r="I199" s="7" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="12" t="n"/>
@@ -4004,6 +4206,7 @@
       <c r="F200" s="8" t="n"/>
       <c r="G200" s="7" t="n"/>
       <c r="H200" s="7" t="n"/>
+      <c r="I200" s="7" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="12" t="n"/>
@@ -4020,6 +4223,7 @@
       <c r="F201" s="8" t="n"/>
       <c r="G201" s="7" t="n"/>
       <c r="H201" s="7" t="n"/>
+      <c r="I201" s="7" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="12" t="n"/>
@@ -4036,6 +4240,7 @@
       <c r="F202" s="8" t="n"/>
       <c r="G202" s="7" t="n"/>
       <c r="H202" s="7" t="n"/>
+      <c r="I202" s="7" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="12" t="n"/>
@@ -4052,6 +4257,7 @@
       <c r="F203" s="8" t="n"/>
       <c r="G203" s="7" t="n"/>
       <c r="H203" s="7" t="n"/>
+      <c r="I203" s="7" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="12" t="n"/>
@@ -4068,6 +4274,7 @@
       <c r="F204" s="8" t="n"/>
       <c r="G204" s="7" t="n"/>
       <c r="H204" s="7" t="n"/>
+      <c r="I204" s="7" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="12" t="n"/>
@@ -4084,6 +4291,7 @@
       <c r="F205" s="8" t="n"/>
       <c r="G205" s="7" t="n"/>
       <c r="H205" s="7" t="n"/>
+      <c r="I205" s="7" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="12" t="n"/>
@@ -4100,6 +4308,7 @@
       <c r="F206" s="8" t="n"/>
       <c r="G206" s="7" t="n"/>
       <c r="H206" s="7" t="n"/>
+      <c r="I206" s="7" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="12" t="n"/>
@@ -4116,6 +4325,7 @@
       <c r="F207" s="8" t="n"/>
       <c r="G207" s="7" t="n"/>
       <c r="H207" s="7" t="n"/>
+      <c r="I207" s="7" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="12" t="n"/>
@@ -4132,6 +4342,7 @@
       <c r="F208" s="8" t="n"/>
       <c r="G208" s="7" t="n"/>
       <c r="H208" s="7" t="n"/>
+      <c r="I208" s="7" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="12" t="n"/>
@@ -4148,6 +4359,7 @@
       <c r="F209" s="8" t="n"/>
       <c r="G209" s="7" t="n"/>
       <c r="H209" s="7" t="n"/>
+      <c r="I209" s="7" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="12" t="n"/>
@@ -4164,6 +4376,7 @@
       <c r="F210" s="8" t="n"/>
       <c r="G210" s="7" t="n"/>
       <c r="H210" s="7" t="n"/>
+      <c r="I210" s="7" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="12" t="n"/>
@@ -4180,6 +4393,7 @@
       <c r="F211" s="8" t="n"/>
       <c r="G211" s="7" t="n"/>
       <c r="H211" s="7" t="n"/>
+      <c r="I211" s="7" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="12" t="n"/>
@@ -4196,6 +4410,7 @@
       <c r="F212" s="8" t="n"/>
       <c r="G212" s="7" t="n"/>
       <c r="H212" s="7" t="n"/>
+      <c r="I212" s="7" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="12" t="n"/>
@@ -4212,6 +4427,7 @@
       <c r="F213" s="8" t="n"/>
       <c r="G213" s="7" t="n"/>
       <c r="H213" s="7" t="n"/>
+      <c r="I213" s="7" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="12" t="n"/>
@@ -4228,6 +4444,7 @@
       <c r="F214" s="8" t="n"/>
       <c r="G214" s="7" t="n"/>
       <c r="H214" s="7" t="n"/>
+      <c r="I214" s="7" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="12" t="n"/>
@@ -4244,6 +4461,7 @@
       <c r="F215" s="8" t="n"/>
       <c r="G215" s="7" t="n"/>
       <c r="H215" s="7" t="n"/>
+      <c r="I215" s="7" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="12" t="n"/>
@@ -4260,6 +4478,7 @@
       <c r="F216" s="8" t="n"/>
       <c r="G216" s="7" t="n"/>
       <c r="H216" s="7" t="n"/>
+      <c r="I216" s="7" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="12" t="n"/>
@@ -4276,6 +4495,7 @@
       <c r="F217" s="8" t="n"/>
       <c r="G217" s="7" t="n"/>
       <c r="H217" s="7" t="n"/>
+      <c r="I217" s="7" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="12" t="n"/>
@@ -4292,6 +4512,7 @@
       <c r="F218" s="8" t="n"/>
       <c r="G218" s="7" t="n"/>
       <c r="H218" s="7" t="n"/>
+      <c r="I218" s="7" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="12" t="n"/>
@@ -4308,6 +4529,7 @@
       <c r="F219" s="8" t="n"/>
       <c r="G219" s="7" t="n"/>
       <c r="H219" s="7" t="n"/>
+      <c r="I219" s="7" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="12" t="n"/>
@@ -4324,6 +4546,7 @@
       <c r="F220" s="8" t="n"/>
       <c r="G220" s="7" t="n"/>
       <c r="H220" s="7" t="n"/>
+      <c r="I220" s="7" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="12" t="n"/>
@@ -4340,6 +4563,7 @@
       <c r="F221" s="8" t="n"/>
       <c r="G221" s="7" t="n"/>
       <c r="H221" s="7" t="n"/>
+      <c r="I221" s="7" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="12" t="n"/>
@@ -4356,6 +4580,7 @@
       <c r="F222" s="8" t="n"/>
       <c r="G222" s="7" t="n"/>
       <c r="H222" s="7" t="n"/>
+      <c r="I222" s="7" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="12" t="n"/>
@@ -4372,6 +4597,7 @@
       <c r="F223" s="8" t="n"/>
       <c r="G223" s="7" t="n"/>
       <c r="H223" s="7" t="n"/>
+      <c r="I223" s="7" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="12" t="n"/>
@@ -4388,6 +4614,7 @@
       <c r="F224" s="8" t="n"/>
       <c r="G224" s="7" t="n"/>
       <c r="H224" s="7" t="n"/>
+      <c r="I224" s="7" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="12" t="n"/>
@@ -4404,6 +4631,7 @@
       <c r="F225" s="8" t="n"/>
       <c r="G225" s="7" t="n"/>
       <c r="H225" s="7" t="n"/>
+      <c r="I225" s="7" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="12" t="n"/>
@@ -4420,6 +4648,7 @@
       <c r="F226" s="8" t="n"/>
       <c r="G226" s="7" t="n"/>
       <c r="H226" s="7" t="n"/>
+      <c r="I226" s="7" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="12" t="n"/>
@@ -4436,6 +4665,7 @@
       <c r="F227" s="8" t="n"/>
       <c r="G227" s="7" t="n"/>
       <c r="H227" s="7" t="n"/>
+      <c r="I227" s="7" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="12" t="n"/>
@@ -4452,6 +4682,7 @@
       <c r="F228" s="8" t="n"/>
       <c r="G228" s="7" t="n"/>
       <c r="H228" s="7" t="n"/>
+      <c r="I228" s="7" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="12" t="n"/>
@@ -4468,6 +4699,7 @@
       <c r="F229" s="8" t="n"/>
       <c r="G229" s="7" t="n"/>
       <c r="H229" s="7" t="n"/>
+      <c r="I229" s="7" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="12" t="n"/>
@@ -4484,6 +4716,7 @@
       <c r="F230" s="8" t="n"/>
       <c r="G230" s="7" t="n"/>
       <c r="H230" s="7" t="n"/>
+      <c r="I230" s="7" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="12" t="n"/>
@@ -4500,6 +4733,7 @@
       <c r="F231" s="8" t="n"/>
       <c r="G231" s="7" t="n"/>
       <c r="H231" s="7" t="n"/>
+      <c r="I231" s="7" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="12" t="n"/>
@@ -4516,6 +4750,7 @@
       <c r="F232" s="8" t="n"/>
       <c r="G232" s="7" t="n"/>
       <c r="H232" s="7" t="n"/>
+      <c r="I232" s="7" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="12" t="n"/>
@@ -4532,6 +4767,7 @@
       <c r="F233" s="8" t="n"/>
       <c r="G233" s="7" t="n"/>
       <c r="H233" s="7" t="n"/>
+      <c r="I233" s="7" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="12" t="n"/>
@@ -4548,6 +4784,7 @@
       <c r="F234" s="8" t="n"/>
       <c r="G234" s="7" t="n"/>
       <c r="H234" s="7" t="n"/>
+      <c r="I234" s="7" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="12" t="n"/>
@@ -4564,6 +4801,7 @@
       <c r="F235" s="8" t="n"/>
       <c r="G235" s="7" t="n"/>
       <c r="H235" s="7" t="n"/>
+      <c r="I235" s="7" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="12" t="n"/>
@@ -4580,6 +4818,7 @@
       <c r="F236" s="8" t="n"/>
       <c r="G236" s="7" t="n"/>
       <c r="H236" s="7" t="n"/>
+      <c r="I236" s="7" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="12" t="n"/>
@@ -4596,6 +4835,7 @@
       <c r="F237" s="8" t="n"/>
       <c r="G237" s="7" t="n"/>
       <c r="H237" s="7" t="n"/>
+      <c r="I237" s="7" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="12" t="n"/>
@@ -4612,6 +4852,7 @@
       <c r="F238" s="8" t="n"/>
       <c r="G238" s="7" t="n"/>
       <c r="H238" s="7" t="n"/>
+      <c r="I238" s="7" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="12" t="n"/>
@@ -4628,6 +4869,7 @@
       <c r="F239" s="8" t="n"/>
       <c r="G239" s="7" t="n"/>
       <c r="H239" s="7" t="n"/>
+      <c r="I239" s="7" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="12" t="n"/>
@@ -4644,6 +4886,7 @@
       <c r="F240" s="8" t="n"/>
       <c r="G240" s="7" t="n"/>
       <c r="H240" s="7" t="n"/>
+      <c r="I240" s="7" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="12" t="n"/>
@@ -4660,6 +4903,7 @@
       <c r="F241" s="8" t="n"/>
       <c r="G241" s="7" t="n"/>
       <c r="H241" s="7" t="n"/>
+      <c r="I241" s="7" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="12" t="n"/>
@@ -4676,6 +4920,7 @@
       <c r="F242" s="8" t="n"/>
       <c r="G242" s="7" t="n"/>
       <c r="H242" s="7" t="n"/>
+      <c r="I242" s="7" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="12" t="n"/>
@@ -4692,6 +4937,7 @@
       <c r="F243" s="8" t="n"/>
       <c r="G243" s="7" t="n"/>
       <c r="H243" s="7" t="n"/>
+      <c r="I243" s="7" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="12" t="n"/>
@@ -4708,6 +4954,7 @@
       <c r="F244" s="8" t="n"/>
       <c r="G244" s="7" t="n"/>
       <c r="H244" s="7" t="n"/>
+      <c r="I244" s="7" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="12" t="n"/>
@@ -4724,6 +4971,7 @@
       <c r="F245" s="8" t="n"/>
       <c r="G245" s="7" t="n"/>
       <c r="H245" s="7" t="n"/>
+      <c r="I245" s="7" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="12" t="n"/>
@@ -4740,6 +4988,7 @@
       <c r="F246" s="8" t="n"/>
       <c r="G246" s="7" t="n"/>
       <c r="H246" s="7" t="n"/>
+      <c r="I246" s="7" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="12" t="n"/>
@@ -4756,6 +5005,7 @@
       <c r="F247" s="8" t="n"/>
       <c r="G247" s="7" t="n"/>
       <c r="H247" s="7" t="n"/>
+      <c r="I247" s="7" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="12" t="n"/>
@@ -4772,6 +5022,7 @@
       <c r="F248" s="8" t="n"/>
       <c r="G248" s="7" t="n"/>
       <c r="H248" s="7" t="n"/>
+      <c r="I248" s="7" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="12" t="n"/>
@@ -4788,6 +5039,7 @@
       <c r="F249" s="8" t="n"/>
       <c r="G249" s="7" t="n"/>
       <c r="H249" s="7" t="n"/>
+      <c r="I249" s="7" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="12" t="n"/>
@@ -4804,6 +5056,7 @@
       <c r="F250" s="8" t="n"/>
       <c r="G250" s="7" t="n"/>
       <c r="H250" s="7" t="n"/>
+      <c r="I250" s="7" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="12" t="n"/>
@@ -4820,6 +5073,7 @@
       <c r="F251" s="8" t="n"/>
       <c r="G251" s="7" t="n"/>
       <c r="H251" s="7" t="n"/>
+      <c r="I251" s="7" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="12" t="n"/>
@@ -4836,6 +5090,7 @@
       <c r="F252" s="8" t="n"/>
       <c r="G252" s="7" t="n"/>
       <c r="H252" s="7" t="n"/>
+      <c r="I252" s="7" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="12" t="n"/>
@@ -4852,6 +5107,7 @@
       <c r="F253" s="8" t="n"/>
       <c r="G253" s="7" t="n"/>
       <c r="H253" s="7" t="n"/>
+      <c r="I253" s="7" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="12" t="n"/>
@@ -4868,6 +5124,7 @@
       <c r="F254" s="8" t="n"/>
       <c r="G254" s="7" t="n"/>
       <c r="H254" s="7" t="n"/>
+      <c r="I254" s="7" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="12" t="n"/>
@@ -4884,6 +5141,7 @@
       <c r="F255" s="8" t="n"/>
       <c r="G255" s="7" t="n"/>
       <c r="H255" s="7" t="n"/>
+      <c r="I255" s="7" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="12" t="n"/>
@@ -4900,6 +5158,7 @@
       <c r="F256" s="8" t="n"/>
       <c r="G256" s="7" t="n"/>
       <c r="H256" s="7" t="n"/>
+      <c r="I256" s="7" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="12" t="n"/>
@@ -4916,6 +5175,7 @@
       <c r="F257" s="8" t="n"/>
       <c r="G257" s="7" t="n"/>
       <c r="H257" s="7" t="n"/>
+      <c r="I257" s="7" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="12" t="n"/>
@@ -4932,6 +5192,7 @@
       <c r="F258" s="8" t="n"/>
       <c r="G258" s="7" t="n"/>
       <c r="H258" s="7" t="n"/>
+      <c r="I258" s="7" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="12" t="n"/>
@@ -4948,6 +5209,7 @@
       <c r="F259" s="8" t="n"/>
       <c r="G259" s="7" t="n"/>
       <c r="H259" s="7" t="n"/>
+      <c r="I259" s="7" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="12" t="n"/>
@@ -4964,6 +5226,7 @@
       <c r="F260" s="8" t="n"/>
       <c r="G260" s="7" t="n"/>
       <c r="H260" s="7" t="n"/>
+      <c r="I260" s="7" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="12" t="n"/>
@@ -4980,6 +5243,7 @@
       <c r="F261" s="8" t="n"/>
       <c r="G261" s="7" t="n"/>
       <c r="H261" s="7" t="n"/>
+      <c r="I261" s="7" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="12" t="n"/>
@@ -4996,6 +5260,7 @@
       <c r="F262" s="8" t="n"/>
       <c r="G262" s="7" t="n"/>
       <c r="H262" s="7" t="n"/>
+      <c r="I262" s="7" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="12" t="n"/>
@@ -5012,6 +5277,7 @@
       <c r="F263" s="8" t="n"/>
       <c r="G263" s="7" t="n"/>
       <c r="H263" s="7" t="n"/>
+      <c r="I263" s="7" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="12" t="n"/>
@@ -5028,6 +5294,7 @@
       <c r="F264" s="8" t="n"/>
       <c r="G264" s="7" t="n"/>
       <c r="H264" s="7" t="n"/>
+      <c r="I264" s="7" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="12" t="n"/>
@@ -5044,6 +5311,7 @@
       <c r="F265" s="8" t="n"/>
       <c r="G265" s="7" t="n"/>
       <c r="H265" s="7" t="n"/>
+      <c r="I265" s="7" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="12" t="n"/>
@@ -5060,6 +5328,7 @@
       <c r="F266" s="8" t="n"/>
       <c r="G266" s="7" t="n"/>
       <c r="H266" s="7" t="n"/>
+      <c r="I266" s="7" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="12" t="n"/>
@@ -5076,6 +5345,7 @@
       <c r="F267" s="8" t="n"/>
       <c r="G267" s="7" t="n"/>
       <c r="H267" s="7" t="n"/>
+      <c r="I267" s="7" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="12" t="n"/>
@@ -5092,6 +5362,7 @@
       <c r="F268" s="8" t="n"/>
       <c r="G268" s="7" t="n"/>
       <c r="H268" s="7" t="n"/>
+      <c r="I268" s="7" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="12" t="n"/>
@@ -5108,6 +5379,7 @@
       <c r="F269" s="8" t="n"/>
       <c r="G269" s="7" t="n"/>
       <c r="H269" s="7" t="n"/>
+      <c r="I269" s="7" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="12" t="n"/>
@@ -5124,6 +5396,7 @@
       <c r="F270" s="8" t="n"/>
       <c r="G270" s="7" t="n"/>
       <c r="H270" s="7" t="n"/>
+      <c r="I270" s="7" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="12" t="n"/>
@@ -5140,6 +5413,7 @@
       <c r="F271" s="8" t="n"/>
       <c r="G271" s="7" t="n"/>
       <c r="H271" s="7" t="n"/>
+      <c r="I271" s="7" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="12" t="n"/>
@@ -5156,6 +5430,7 @@
       <c r="F272" s="8" t="n"/>
       <c r="G272" s="7" t="n"/>
       <c r="H272" s="7" t="n"/>
+      <c r="I272" s="7" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="12" t="n"/>
@@ -5172,6 +5447,7 @@
       <c r="F273" s="8" t="n"/>
       <c r="G273" s="7" t="n"/>
       <c r="H273" s="7" t="n"/>
+      <c r="I273" s="7" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="12" t="n"/>
@@ -5188,6 +5464,7 @@
       <c r="F274" s="8" t="n"/>
       <c r="G274" s="7" t="n"/>
       <c r="H274" s="7" t="n"/>
+      <c r="I274" s="7" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="12" t="n"/>
@@ -5204,6 +5481,7 @@
       <c r="F275" s="8" t="n"/>
       <c r="G275" s="7" t="n"/>
       <c r="H275" s="7" t="n"/>
+      <c r="I275" s="7" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="12" t="n"/>
@@ -5220,6 +5498,7 @@
       <c r="F276" s="8" t="n"/>
       <c r="G276" s="7" t="n"/>
       <c r="H276" s="7" t="n"/>
+      <c r="I276" s="7" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="12" t="n"/>
@@ -5236,6 +5515,7 @@
       <c r="F277" s="8" t="n"/>
       <c r="G277" s="7" t="n"/>
       <c r="H277" s="7" t="n"/>
+      <c r="I277" s="7" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="12" t="n"/>
@@ -5252,6 +5532,7 @@
       <c r="F278" s="8" t="n"/>
       <c r="G278" s="7" t="n"/>
       <c r="H278" s="7" t="n"/>
+      <c r="I278" s="7" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="12" t="n"/>
@@ -5268,6 +5549,7 @@
       <c r="F279" s="8" t="n"/>
       <c r="G279" s="7" t="n"/>
       <c r="H279" s="7" t="n"/>
+      <c r="I279" s="7" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="12" t="n"/>
@@ -5284,6 +5566,7 @@
       <c r="F280" s="8" t="n"/>
       <c r="G280" s="7" t="n"/>
       <c r="H280" s="7" t="n"/>
+      <c r="I280" s="7" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="12" t="n"/>
@@ -5300,6 +5583,7 @@
       <c r="F281" s="8" t="n"/>
       <c r="G281" s="7" t="n"/>
       <c r="H281" s="7" t="n"/>
+      <c r="I281" s="7" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="12" t="n"/>
@@ -5316,6 +5600,7 @@
       <c r="F282" s="8" t="n"/>
       <c r="G282" s="7" t="n"/>
       <c r="H282" s="7" t="n"/>
+      <c r="I282" s="7" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="12" t="n"/>
@@ -5332,6 +5617,7 @@
       <c r="F283" s="8" t="n"/>
       <c r="G283" s="7" t="n"/>
       <c r="H283" s="7" t="n"/>
+      <c r="I283" s="7" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="12" t="n"/>
@@ -5348,6 +5634,7 @@
       <c r="F284" s="8" t="n"/>
       <c r="G284" s="7" t="n"/>
       <c r="H284" s="7" t="n"/>
+      <c r="I284" s="7" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="12" t="n"/>
@@ -5364,6 +5651,7 @@
       <c r="F285" s="8" t="n"/>
       <c r="G285" s="7" t="n"/>
       <c r="H285" s="7" t="n"/>
+      <c r="I285" s="7" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="12" t="n"/>
@@ -5380,6 +5668,7 @@
       <c r="F286" s="8" t="n"/>
       <c r="G286" s="7" t="n"/>
       <c r="H286" s="7" t="n"/>
+      <c r="I286" s="7" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="12" t="n"/>
@@ -5396,6 +5685,7 @@
       <c r="F287" s="8" t="n"/>
       <c r="G287" s="7" t="n"/>
       <c r="H287" s="7" t="n"/>
+      <c r="I287" s="7" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="12" t="n"/>
@@ -5412,6 +5702,7 @@
       <c r="F288" s="8" t="n"/>
       <c r="G288" s="7" t="n"/>
       <c r="H288" s="7" t="n"/>
+      <c r="I288" s="7" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="12" t="n"/>
@@ -5428,6 +5719,7 @@
       <c r="F289" s="8" t="n"/>
       <c r="G289" s="7" t="n"/>
       <c r="H289" s="7" t="n"/>
+      <c r="I289" s="7" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="12" t="n"/>
@@ -5444,6 +5736,7 @@
       <c r="F290" s="8" t="n"/>
       <c r="G290" s="7" t="n"/>
       <c r="H290" s="7" t="n"/>
+      <c r="I290" s="7" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="12" t="n"/>
@@ -5460,6 +5753,7 @@
       <c r="F291" s="8" t="n"/>
       <c r="G291" s="7" t="n"/>
       <c r="H291" s="7" t="n"/>
+      <c r="I291" s="7" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="12" t="n"/>
@@ -5476,6 +5770,7 @@
       <c r="F292" s="8" t="n"/>
       <c r="G292" s="7" t="n"/>
       <c r="H292" s="7" t="n"/>
+      <c r="I292" s="7" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="12" t="n"/>
@@ -5492,6 +5787,7 @@
       <c r="F293" s="8" t="n"/>
       <c r="G293" s="7" t="n"/>
       <c r="H293" s="7" t="n"/>
+      <c r="I293" s="7" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="12" t="n"/>
@@ -5508,6 +5804,7 @@
       <c r="F294" s="8" t="n"/>
       <c r="G294" s="7" t="n"/>
       <c r="H294" s="7" t="n"/>
+      <c r="I294" s="7" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="12" t="n"/>
@@ -5524,6 +5821,7 @@
       <c r="F295" s="8" t="n"/>
       <c r="G295" s="7" t="n"/>
       <c r="H295" s="7" t="n"/>
+      <c r="I295" s="7" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="12" t="n"/>
@@ -5540,6 +5838,7 @@
       <c r="F296" s="8" t="n"/>
       <c r="G296" s="7" t="n"/>
       <c r="H296" s="7" t="n"/>
+      <c r="I296" s="7" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="12" t="n"/>
@@ -5556,6 +5855,7 @@
       <c r="F297" s="8" t="n"/>
       <c r="G297" s="7" t="n"/>
       <c r="H297" s="7" t="n"/>
+      <c r="I297" s="7" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="12" t="n"/>
@@ -5572,6 +5872,7 @@
       <c r="F298" s="8" t="n"/>
       <c r="G298" s="7" t="n"/>
       <c r="H298" s="7" t="n"/>
+      <c r="I298" s="7" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="12" t="n"/>
@@ -5588,6 +5889,7 @@
       <c r="F299" s="8" t="n"/>
       <c r="G299" s="7" t="n"/>
       <c r="H299" s="7" t="n"/>
+      <c r="I299" s="7" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="12" t="n"/>
@@ -5604,6 +5906,7 @@
       <c r="F300" s="8" t="n"/>
       <c r="G300" s="7" t="n"/>
       <c r="H300" s="7" t="n"/>
+      <c r="I300" s="7" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="12" t="n"/>
@@ -5620,6 +5923,7 @@
       <c r="F301" s="8" t="n"/>
       <c r="G301" s="7" t="n"/>
       <c r="H301" s="7" t="n"/>
+      <c r="I301" s="7" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="12" t="n"/>
@@ -5636,6 +5940,7 @@
       <c r="F302" s="8" t="n"/>
       <c r="G302" s="7" t="n"/>
       <c r="H302" s="7" t="n"/>
+      <c r="I302" s="7" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="12" t="n"/>
@@ -5652,6 +5957,7 @@
       <c r="F303" s="8" t="n"/>
       <c r="G303" s="7" t="n"/>
       <c r="H303" s="7" t="n"/>
+      <c r="I303" s="7" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="12" t="n"/>
@@ -5668,6 +5974,7 @@
       <c r="F304" s="8" t="n"/>
       <c r="G304" s="7" t="n"/>
       <c r="H304" s="7" t="n"/>
+      <c r="I304" s="7" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="12" t="n"/>
@@ -5684,6 +5991,7 @@
       <c r="F305" s="8" t="n"/>
       <c r="G305" s="7" t="n"/>
       <c r="H305" s="7" t="n"/>
+      <c r="I305" s="7" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="12" t="n"/>
@@ -5700,6 +6008,7 @@
       <c r="F306" s="8" t="n"/>
       <c r="G306" s="7" t="n"/>
       <c r="H306" s="7" t="n"/>
+      <c r="I306" s="7" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="12" t="n"/>
@@ -5716,6 +6025,7 @@
       <c r="F307" s="8" t="n"/>
       <c r="G307" s="7" t="n"/>
       <c r="H307" s="7" t="n"/>
+      <c r="I307" s="7" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="12" t="n"/>
@@ -5732,6 +6042,7 @@
       <c r="F308" s="8" t="n"/>
       <c r="G308" s="7" t="n"/>
       <c r="H308" s="7" t="n"/>
+      <c r="I308" s="7" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="12" t="n"/>
@@ -5748,6 +6059,7 @@
       <c r="F309" s="8" t="n"/>
       <c r="G309" s="7" t="n"/>
       <c r="H309" s="7" t="n"/>
+      <c r="I309" s="7" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="12" t="n"/>
@@ -5764,6 +6076,7 @@
       <c r="F310" s="8" t="n"/>
       <c r="G310" s="7" t="n"/>
       <c r="H310" s="7" t="n"/>
+      <c r="I310" s="7" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="12" t="n"/>
@@ -5780,6 +6093,7 @@
       <c r="F311" s="8" t="n"/>
       <c r="G311" s="7" t="n"/>
       <c r="H311" s="7" t="n"/>
+      <c r="I311" s="7" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="12" t="n"/>
@@ -5796,6 +6110,7 @@
       <c r="F312" s="8" t="n"/>
       <c r="G312" s="7" t="n"/>
       <c r="H312" s="7" t="n"/>
+      <c r="I312" s="7" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="12" t="n"/>
@@ -5812,6 +6127,7 @@
       <c r="F313" s="8" t="n"/>
       <c r="G313" s="7" t="n"/>
       <c r="H313" s="7" t="n"/>
+      <c r="I313" s="7" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="12" t="n"/>
@@ -5828,6 +6144,7 @@
       <c r="F314" s="8" t="n"/>
       <c r="G314" s="7" t="n"/>
       <c r="H314" s="7" t="n"/>
+      <c r="I314" s="7" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="12" t="n"/>
@@ -5844,6 +6161,7 @@
       <c r="F315" s="8" t="n"/>
       <c r="G315" s="7" t="n"/>
       <c r="H315" s="7" t="n"/>
+      <c r="I315" s="7" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="12" t="n"/>
@@ -5860,6 +6178,7 @@
       <c r="F316" s="8" t="n"/>
       <c r="G316" s="7" t="n"/>
       <c r="H316" s="7" t="n"/>
+      <c r="I316" s="7" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="12" t="n"/>
@@ -5876,6 +6195,7 @@
       <c r="F317" s="8" t="n"/>
       <c r="G317" s="7" t="n"/>
       <c r="H317" s="7" t="n"/>
+      <c r="I317" s="7" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="12" t="n"/>
@@ -5892,6 +6212,7 @@
       <c r="F318" s="8" t="n"/>
       <c r="G318" s="7" t="n"/>
       <c r="H318" s="7" t="n"/>
+      <c r="I318" s="7" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="12" t="n"/>
@@ -5908,6 +6229,7 @@
       <c r="F319" s="8" t="n"/>
       <c r="G319" s="7" t="n"/>
       <c r="H319" s="7" t="n"/>
+      <c r="I319" s="7" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="12" t="n"/>
@@ -5924,6 +6246,7 @@
       <c r="F320" s="8" t="n"/>
       <c r="G320" s="7" t="n"/>
       <c r="H320" s="7" t="n"/>
+      <c r="I320" s="7" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="12" t="n"/>
@@ -5940,6 +6263,7 @@
       <c r="F321" s="8" t="n"/>
       <c r="G321" s="7" t="n"/>
       <c r="H321" s="7" t="n"/>
+      <c r="I321" s="7" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="12" t="n"/>
@@ -5956,6 +6280,7 @@
       <c r="F322" s="8" t="n"/>
       <c r="G322" s="7" t="n"/>
       <c r="H322" s="7" t="n"/>
+      <c r="I322" s="7" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="12" t="n"/>
@@ -5972,6 +6297,7 @@
       <c r="F323" s="8" t="n"/>
       <c r="G323" s="7" t="n"/>
       <c r="H323" s="7" t="n"/>
+      <c r="I323" s="7" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="12" t="n"/>
@@ -5988,6 +6314,7 @@
       <c r="F324" s="8" t="n"/>
       <c r="G324" s="7" t="n"/>
       <c r="H324" s="7" t="n"/>
+      <c r="I324" s="7" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="12" t="n"/>
@@ -6004,6 +6331,7 @@
       <c r="F325" s="8" t="n"/>
       <c r="G325" s="7" t="n"/>
       <c r="H325" s="7" t="n"/>
+      <c r="I325" s="7" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="12" t="n"/>
@@ -6020,6 +6348,7 @@
       <c r="F326" s="8" t="n"/>
       <c r="G326" s="7" t="n"/>
       <c r="H326" s="7" t="n"/>
+      <c r="I326" s="7" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="12" t="n"/>
@@ -6036,6 +6365,7 @@
       <c r="F327" s="8" t="n"/>
       <c r="G327" s="7" t="n"/>
       <c r="H327" s="7" t="n"/>
+      <c r="I327" s="7" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="12" t="n"/>
@@ -6052,6 +6382,7 @@
       <c r="F328" s="8" t="n"/>
       <c r="G328" s="7" t="n"/>
       <c r="H328" s="7" t="n"/>
+      <c r="I328" s="7" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="12" t="n"/>
@@ -6068,6 +6399,7 @@
       <c r="F329" s="8" t="n"/>
       <c r="G329" s="7" t="n"/>
       <c r="H329" s="7" t="n"/>
+      <c r="I329" s="7" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="12" t="n"/>
@@ -6084,6 +6416,7 @@
       <c r="F330" s="8" t="n"/>
       <c r="G330" s="7" t="n"/>
       <c r="H330" s="7" t="n"/>
+      <c r="I330" s="7" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="12" t="n"/>
@@ -6100,6 +6433,7 @@
       <c r="F331" s="8" t="n"/>
       <c r="G331" s="7" t="n"/>
       <c r="H331" s="7" t="n"/>
+      <c r="I331" s="7" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="12" t="n"/>
@@ -6116,6 +6450,7 @@
       <c r="F332" s="8" t="n"/>
       <c r="G332" s="7" t="n"/>
       <c r="H332" s="7" t="n"/>
+      <c r="I332" s="7" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="12" t="n"/>
@@ -6132,6 +6467,7 @@
       <c r="F333" s="8" t="n"/>
       <c r="G333" s="7" t="n"/>
       <c r="H333" s="7" t="n"/>
+      <c r="I333" s="7" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="12" t="n"/>
@@ -6148,6 +6484,7 @@
       <c r="F334" s="8" t="n"/>
       <c r="G334" s="7" t="n"/>
       <c r="H334" s="7" t="n"/>
+      <c r="I334" s="7" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="12" t="n"/>
@@ -6164,6 +6501,7 @@
       <c r="F335" s="8" t="n"/>
       <c r="G335" s="7" t="n"/>
       <c r="H335" s="7" t="n"/>
+      <c r="I335" s="7" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="12" t="n"/>
@@ -6180,6 +6518,7 @@
       <c r="F336" s="8" t="n"/>
       <c r="G336" s="7" t="n"/>
       <c r="H336" s="7" t="n"/>
+      <c r="I336" s="7" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="12" t="n"/>
@@ -6196,6 +6535,7 @@
       <c r="F337" s="8" t="n"/>
       <c r="G337" s="7" t="n"/>
       <c r="H337" s="7" t="n"/>
+      <c r="I337" s="7" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="12" t="n"/>
@@ -6212,6 +6552,7 @@
       <c r="F338" s="8" t="n"/>
       <c r="G338" s="7" t="n"/>
       <c r="H338" s="7" t="n"/>
+      <c r="I338" s="7" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="12" t="n"/>
@@ -6228,6 +6569,7 @@
       <c r="F339" s="8" t="n"/>
       <c r="G339" s="7" t="n"/>
       <c r="H339" s="7" t="n"/>
+      <c r="I339" s="7" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="12" t="n"/>
@@ -6244,6 +6586,7 @@
       <c r="F340" s="8" t="n"/>
       <c r="G340" s="7" t="n"/>
       <c r="H340" s="7" t="n"/>
+      <c r="I340" s="7" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="12" t="n"/>
@@ -6260,6 +6603,7 @@
       <c r="F341" s="8" t="n"/>
       <c r="G341" s="7" t="n"/>
       <c r="H341" s="7" t="n"/>
+      <c r="I341" s="7" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="12" t="n"/>
@@ -6276,6 +6620,7 @@
       <c r="F342" s="8" t="n"/>
       <c r="G342" s="7" t="n"/>
       <c r="H342" s="7" t="n"/>
+      <c r="I342" s="7" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="12" t="n"/>
@@ -6292,6 +6637,7 @@
       <c r="F343" s="8" t="n"/>
       <c r="G343" s="7" t="n"/>
       <c r="H343" s="7" t="n"/>
+      <c r="I343" s="7" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="12" t="n"/>
@@ -6308,6 +6654,7 @@
       <c r="F344" s="8" t="n"/>
       <c r="G344" s="7" t="n"/>
       <c r="H344" s="7" t="n"/>
+      <c r="I344" s="7" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="12" t="n"/>
@@ -6324,6 +6671,7 @@
       <c r="F345" s="8" t="n"/>
       <c r="G345" s="7" t="n"/>
       <c r="H345" s="7" t="n"/>
+      <c r="I345" s="7" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="12" t="n"/>
@@ -6340,6 +6688,7 @@
       <c r="F346" s="8" t="n"/>
       <c r="G346" s="7" t="n"/>
       <c r="H346" s="7" t="n"/>
+      <c r="I346" s="7" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="12" t="n"/>
@@ -6356,6 +6705,7 @@
       <c r="F347" s="8" t="n"/>
       <c r="G347" s="7" t="n"/>
       <c r="H347" s="7" t="n"/>
+      <c r="I347" s="7" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="12" t="n"/>
@@ -6372,6 +6722,7 @@
       <c r="F348" s="8" t="n"/>
       <c r="G348" s="7" t="n"/>
       <c r="H348" s="7" t="n"/>
+      <c r="I348" s="7" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="12" t="n"/>
@@ -6388,6 +6739,7 @@
       <c r="F349" s="8" t="n"/>
       <c r="G349" s="7" t="n"/>
       <c r="H349" s="7" t="n"/>
+      <c r="I349" s="7" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="12" t="n"/>
@@ -6404,6 +6756,7 @@
       <c r="F350" s="8" t="n"/>
       <c r="G350" s="7" t="n"/>
       <c r="H350" s="7" t="n"/>
+      <c r="I350" s="7" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="12" t="n"/>
@@ -6420,6 +6773,7 @@
       <c r="F351" s="8" t="n"/>
       <c r="G351" s="7" t="n"/>
       <c r="H351" s="7" t="n"/>
+      <c r="I351" s="7" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="12" t="n"/>
@@ -6436,6 +6790,7 @@
       <c r="F352" s="8" t="n"/>
       <c r="G352" s="7" t="n"/>
       <c r="H352" s="7" t="n"/>
+      <c r="I352" s="7" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="12" t="n"/>
@@ -6452,6 +6807,7 @@
       <c r="F353" s="8" t="n"/>
       <c r="G353" s="7" t="n"/>
       <c r="H353" s="7" t="n"/>
+      <c r="I353" s="7" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="12" t="n"/>
@@ -6468,6 +6824,7 @@
       <c r="F354" s="8" t="n"/>
       <c r="G354" s="7" t="n"/>
       <c r="H354" s="7" t="n"/>
+      <c r="I354" s="7" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="12" t="n"/>
@@ -6484,6 +6841,7 @@
       <c r="F355" s="8" t="n"/>
       <c r="G355" s="7" t="n"/>
       <c r="H355" s="7" t="n"/>
+      <c r="I355" s="7" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="12" t="n"/>
@@ -6500,6 +6858,7 @@
       <c r="F356" s="8" t="n"/>
       <c r="G356" s="7" t="n"/>
       <c r="H356" s="7" t="n"/>
+      <c r="I356" s="7" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="12" t="n"/>
@@ -6516,6 +6875,7 @@
       <c r="F357" s="8" t="n"/>
       <c r="G357" s="7" t="n"/>
       <c r="H357" s="7" t="n"/>
+      <c r="I357" s="7" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="12" t="n"/>
@@ -6532,6 +6892,7 @@
       <c r="F358" s="8" t="n"/>
       <c r="G358" s="7" t="n"/>
       <c r="H358" s="7" t="n"/>
+      <c r="I358" s="7" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="12" t="n"/>
@@ -6548,6 +6909,7 @@
       <c r="F359" s="8" t="n"/>
       <c r="G359" s="7" t="n"/>
       <c r="H359" s="7" t="n"/>
+      <c r="I359" s="7" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="12" t="n"/>
@@ -6564,6 +6926,7 @@
       <c r="F360" s="8" t="n"/>
       <c r="G360" s="7" t="n"/>
       <c r="H360" s="7" t="n"/>
+      <c r="I360" s="7" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="12" t="n"/>
@@ -6580,6 +6943,7 @@
       <c r="F361" s="8" t="n"/>
       <c r="G361" s="7" t="n"/>
       <c r="H361" s="7" t="n"/>
+      <c r="I361" s="7" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="12" t="n"/>
@@ -6596,6 +6960,7 @@
       <c r="F362" s="8" t="n"/>
       <c r="G362" s="7" t="n"/>
       <c r="H362" s="7" t="n"/>
+      <c r="I362" s="7" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="12" t="n"/>
@@ -6612,6 +6977,7 @@
       <c r="F363" s="8" t="n"/>
       <c r="G363" s="7" t="n"/>
       <c r="H363" s="7" t="n"/>
+      <c r="I363" s="7" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="12" t="n"/>
@@ -6628,6 +6994,7 @@
       <c r="F364" s="8" t="n"/>
       <c r="G364" s="7" t="n"/>
       <c r="H364" s="7" t="n"/>
+      <c r="I364" s="7" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="12" t="n"/>
@@ -6644,6 +7011,7 @@
       <c r="F365" s="8" t="n"/>
       <c r="G365" s="7" t="n"/>
       <c r="H365" s="7" t="n"/>
+      <c r="I365" s="7" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="12" t="n"/>
@@ -6660,6 +7028,7 @@
       <c r="F366" s="8" t="n"/>
       <c r="G366" s="7" t="n"/>
       <c r="H366" s="7" t="n"/>
+      <c r="I366" s="7" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="12" t="n"/>
@@ -6676,6 +7045,7 @@
       <c r="F367" s="8" t="n"/>
       <c r="G367" s="7" t="n"/>
       <c r="H367" s="7" t="n"/>
+      <c r="I367" s="7" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="12" t="n"/>
@@ -6692,6 +7062,7 @@
       <c r="F368" s="8" t="n"/>
       <c r="G368" s="7" t="n"/>
       <c r="H368" s="7" t="n"/>
+      <c r="I368" s="7" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="12" t="n"/>
@@ -6708,6 +7079,7 @@
       <c r="F369" s="8" t="n"/>
       <c r="G369" s="7" t="n"/>
       <c r="H369" s="7" t="n"/>
+      <c r="I369" s="7" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="12" t="n"/>
@@ -6724,6 +7096,7 @@
       <c r="F370" s="8" t="n"/>
       <c r="G370" s="7" t="n"/>
       <c r="H370" s="7" t="n"/>
+      <c r="I370" s="7" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="12" t="n"/>
@@ -6740,6 +7113,7 @@
       <c r="F371" s="8" t="n"/>
       <c r="G371" s="7" t="n"/>
       <c r="H371" s="7" t="n"/>
+      <c r="I371" s="7" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="12" t="n"/>
@@ -6756,6 +7130,7 @@
       <c r="F372" s="8" t="n"/>
       <c r="G372" s="7" t="n"/>
       <c r="H372" s="7" t="n"/>
+      <c r="I372" s="7" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="12" t="n"/>
@@ -6772,6 +7147,7 @@
       <c r="F373" s="8" t="n"/>
       <c r="G373" s="7" t="n"/>
       <c r="H373" s="7" t="n"/>
+      <c r="I373" s="7" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="12" t="n"/>
@@ -6788,6 +7164,7 @@
       <c r="F374" s="8" t="n"/>
       <c r="G374" s="7" t="n"/>
       <c r="H374" s="7" t="n"/>
+      <c r="I374" s="7" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="12" t="n"/>
@@ -6804,6 +7181,7 @@
       <c r="F375" s="8" t="n"/>
       <c r="G375" s="7" t="n"/>
       <c r="H375" s="7" t="n"/>
+      <c r="I375" s="7" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="12" t="n"/>
@@ -6820,6 +7198,7 @@
       <c r="F376" s="8" t="n"/>
       <c r="G376" s="7" t="n"/>
       <c r="H376" s="7" t="n"/>
+      <c r="I376" s="7" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="12" t="n"/>
@@ -6836,6 +7215,7 @@
       <c r="F377" s="8" t="n"/>
       <c r="G377" s="7" t="n"/>
       <c r="H377" s="7" t="n"/>
+      <c r="I377" s="7" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="12" t="n"/>
@@ -6852,6 +7232,7 @@
       <c r="F378" s="8" t="n"/>
       <c r="G378" s="7" t="n"/>
       <c r="H378" s="7" t="n"/>
+      <c r="I378" s="7" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="12" t="n"/>
@@ -6868,6 +7249,7 @@
       <c r="F379" s="8" t="n"/>
       <c r="G379" s="7" t="n"/>
       <c r="H379" s="7" t="n"/>
+      <c r="I379" s="7" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="12" t="n"/>
@@ -6884,6 +7266,7 @@
       <c r="F380" s="8" t="n"/>
       <c r="G380" s="7" t="n"/>
       <c r="H380" s="7" t="n"/>
+      <c r="I380" s="7" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="12" t="n"/>
@@ -6900,6 +7283,7 @@
       <c r="F381" s="8" t="n"/>
       <c r="G381" s="7" t="n"/>
       <c r="H381" s="7" t="n"/>
+      <c r="I381" s="7" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="12" t="n"/>
@@ -6916,6 +7300,7 @@
       <c r="F382" s="8" t="n"/>
       <c r="G382" s="7" t="n"/>
       <c r="H382" s="7" t="n"/>
+      <c r="I382" s="7" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="12" t="n"/>
@@ -6932,6 +7317,7 @@
       <c r="F383" s="8" t="n"/>
       <c r="G383" s="7" t="n"/>
       <c r="H383" s="7" t="n"/>
+      <c r="I383" s="7" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="12" t="n"/>
@@ -6948,6 +7334,7 @@
       <c r="F384" s="8" t="n"/>
       <c r="G384" s="7" t="n"/>
       <c r="H384" s="7" t="n"/>
+      <c r="I384" s="7" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="12" t="n"/>
@@ -6964,6 +7351,7 @@
       <c r="F385" s="8" t="n"/>
       <c r="G385" s="7" t="n"/>
       <c r="H385" s="7" t="n"/>
+      <c r="I385" s="7" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="12" t="n"/>
@@ -6980,6 +7368,7 @@
       <c r="F386" s="8" t="n"/>
       <c r="G386" s="7" t="n"/>
       <c r="H386" s="7" t="n"/>
+      <c r="I386" s="7" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="12" t="n"/>
@@ -6996,6 +7385,7 @@
       <c r="F387" s="8" t="n"/>
       <c r="G387" s="7" t="n"/>
       <c r="H387" s="7" t="n"/>
+      <c r="I387" s="7" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="12" t="n"/>
@@ -7012,6 +7402,7 @@
       <c r="F388" s="8" t="n"/>
       <c r="G388" s="7" t="n"/>
       <c r="H388" s="7" t="n"/>
+      <c r="I388" s="7" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="12" t="n"/>
@@ -7028,6 +7419,7 @@
       <c r="F389" s="8" t="n"/>
       <c r="G389" s="7" t="n"/>
       <c r="H389" s="7" t="n"/>
+      <c r="I389" s="7" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="12" t="n"/>
@@ -7044,6 +7436,7 @@
       <c r="F390" s="8" t="n"/>
       <c r="G390" s="7" t="n"/>
       <c r="H390" s="7" t="n"/>
+      <c r="I390" s="7" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="12" t="n"/>
@@ -7060,6 +7453,7 @@
       <c r="F391" s="8" t="n"/>
       <c r="G391" s="7" t="n"/>
       <c r="H391" s="7" t="n"/>
+      <c r="I391" s="7" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="12" t="n"/>
@@ -7076,6 +7470,7 @@
       <c r="F392" s="8" t="n"/>
       <c r="G392" s="7" t="n"/>
       <c r="H392" s="7" t="n"/>
+      <c r="I392" s="7" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="12" t="n"/>
@@ -7092,6 +7487,7 @@
       <c r="F393" s="8" t="n"/>
       <c r="G393" s="7" t="n"/>
       <c r="H393" s="7" t="n"/>
+      <c r="I393" s="7" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="12" t="n"/>
@@ -7108,6 +7504,7 @@
       <c r="F394" s="8" t="n"/>
       <c r="G394" s="7" t="n"/>
       <c r="H394" s="7" t="n"/>
+      <c r="I394" s="7" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="12" t="n"/>
@@ -7124,6 +7521,7 @@
       <c r="F395" s="8" t="n"/>
       <c r="G395" s="7" t="n"/>
       <c r="H395" s="7" t="n"/>
+      <c r="I395" s="7" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="12" t="n"/>
@@ -7140,6 +7538,7 @@
       <c r="F396" s="8" t="n"/>
       <c r="G396" s="7" t="n"/>
       <c r="H396" s="7" t="n"/>
+      <c r="I396" s="7" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="12" t="n"/>
@@ -7156,6 +7555,7 @@
       <c r="F397" s="8" t="n"/>
       <c r="G397" s="7" t="n"/>
       <c r="H397" s="7" t="n"/>
+      <c r="I397" s="7" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="12" t="n"/>
@@ -7172,6 +7572,7 @@
       <c r="F398" s="8" t="n"/>
       <c r="G398" s="7" t="n"/>
       <c r="H398" s="7" t="n"/>
+      <c r="I398" s="7" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="12" t="n"/>
@@ -7188,6 +7589,7 @@
       <c r="F399" s="8" t="n"/>
       <c r="G399" s="7" t="n"/>
       <c r="H399" s="7" t="n"/>
+      <c r="I399" s="7" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="12" t="n"/>
@@ -7204,6 +7606,7 @@
       <c r="F400" s="8" t="n"/>
       <c r="G400" s="7" t="n"/>
       <c r="H400" s="7" t="n"/>
+      <c r="I400" s="7" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="12" t="n"/>
@@ -7220,6 +7623,7 @@
       <c r="F401" s="8" t="n"/>
       <c r="G401" s="7" t="n"/>
       <c r="H401" s="7" t="n"/>
+      <c r="I401" s="7" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="12" t="n"/>
@@ -7236,6 +7640,7 @@
       <c r="F402" s="8" t="n"/>
       <c r="G402" s="7" t="n"/>
       <c r="H402" s="7" t="n"/>
+      <c r="I402" s="7" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="12" t="n"/>
@@ -7252,11 +7657,12 @@
       <c r="F403" s="8" t="n"/>
       <c r="G403" s="7" t="n"/>
       <c r="H403" s="7" t="n"/>
+      <c r="I403" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:E403">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -7283,7 +7689,7 @@
       <formula>AND($A4&lt;&gt;"",$F4="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:H403">
+  <conditionalFormatting sqref="A4:I403">
     <cfRule type="expression" priority="8" dxfId="7">
       <formula>AND($A4&lt;&gt;"",ISEVEN(WEEKNUM($A4,1)))</formula>
     </cfRule>
@@ -10186,13 +10592,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B23"/>
+  <dimension ref="B1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="10" t="inlineStr">
         <is>
@@ -10246,7 +10653,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>7. Foto (opcional): sube la foto a la carpeta de Drive de la agenda (compartida con «Cualquier persona con el enlace») y pega aquí su enlace.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">

</xml_diff>